<commit_message>
Fix formula-text conflict in 01_Loan_Analysis.xlsx: prefix display strings starting with = to prevent openpyxl from treating them as Excel formulas
</commit_message>
<xml_diff>
--- a/rFLA300/chapter-11/01_Loan_Analysis.xlsx
+++ b/rFLA300/chapter-11/01_Loan_Analysis.xlsx
@@ -906,9 +906,10 @@
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
-      <c r="B20" s="19">
-        <f>PMT(rate, nper, pv, [fv], [type])</f>
-        <v/>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> =PMT(rate, nper, pv, [fv], [type])</t>
+        </is>
       </c>
       <c r="C20" s="5" t="inlineStr"/>
     </row>
@@ -1606,9 +1607,10 @@
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="11">
-        <f>CUMIPMT(rate, nper, pv, start_period, end_period, type)   →  returns NEGATIVE</f>
-        <v/>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  =CUMIPMT(rate, nper, pv, start_period, end_period, type)   →  returns NEGATIVE</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -1663,9 +1665,10 @@
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="11">
-        <f>CUMPRINC(rate, nper, pv, start_period, end_period, type)  →  returns NEGATIVE</f>
-        <v/>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  =CUMPRINC(rate, nper, pv, start_period, end_period, type)  →  returns NEGATIVE</t>
+        </is>
       </c>
     </row>
     <row r="24">

</xml_diff>